<commit_message>
Changed lead time to 5 years
</commit_message>
<xml_diff>
--- a/SubRES_TMPL/SubRES_SUP_Hydrogen.xlsx
+++ b/SubRES_TMPL/SubRES_SUP_Hydrogen.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbsul\Documents\GitHub\times-ireland-model\SubRES_TMPL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\21254792\Documents\Git\times-ireland-model\SubRES_TMPL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64455B47-3B87-4E8D-9C48-58217D2EB668}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{423775FA-96C7-4E66-B7BE-222069E18AB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{62F67F8D-DFD4-4ADE-8356-63F780461C4E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{62F67F8D-DFD4-4ADE-8356-63F780461C4E}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="7" r:id="rId1"/>
@@ -1541,20 +1541,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93D8E05A-A755-453F-A2CC-13F04C55B174}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Z99"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="4" width="21.7265625" customWidth="1"/>
-    <col min="5" max="6" width="14.08984375" customWidth="1"/>
-    <col min="7" max="7" width="12.08984375" customWidth="1"/>
-    <col min="8" max="10" width="8.08984375" customWidth="1"/>
-    <col min="11" max="11" width="9.7265625" customWidth="1"/>
-    <col min="12" max="12" width="8.08984375" customWidth="1"/>
+    <col min="1" max="4" width="21.77734375" customWidth="1"/>
+    <col min="5" max="6" width="14.109375" customWidth="1"/>
+    <col min="7" max="7" width="12.109375" customWidth="1"/>
+    <col min="8" max="10" width="8.109375" customWidth="1"/>
+    <col min="11" max="11" width="9.77734375" customWidth="1"/>
+    <col min="12" max="12" width="8.109375" customWidth="1"/>
     <col min="13" max="13" width="10" customWidth="1"/>
-    <col min="14" max="14" width="11.36328125" customWidth="1"/>
-    <col min="15" max="15" width="13.36328125" customWidth="1"/>
+    <col min="14" max="14" width="11.33203125" customWidth="1"/>
+    <col min="15" max="15" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1" s="24"/>
       <c r="B1" s="24"/>
       <c r="C1" s="24"/>
@@ -1582,7 +1582,7 @@
       <c r="Y1" s="25"/>
       <c r="Z1" s="25"/>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A2" s="24"/>
       <c r="B2" s="24"/>
       <c r="C2" s="24"/>
@@ -1610,7 +1610,7 @@
       <c r="Y2" s="25"/>
       <c r="Z2" s="25"/>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A3" s="24"/>
       <c r="B3" s="24"/>
       <c r="C3" s="24"/>
@@ -1638,7 +1638,7 @@
       <c r="Y3" s="25"/>
       <c r="Z3" s="25"/>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4" s="24"/>
       <c r="B4" s="24"/>
       <c r="C4" s="24"/>
@@ -1666,7 +1666,7 @@
       <c r="Y4" s="25"/>
       <c r="Z4" s="25"/>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5" s="24"/>
       <c r="B5" s="24"/>
       <c r="C5" s="24"/>
@@ -1694,7 +1694,7 @@
       <c r="Y5" s="25"/>
       <c r="Z5" s="25"/>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6" s="24"/>
       <c r="B6" s="24"/>
       <c r="C6" s="24"/>
@@ -1722,7 +1722,7 @@
       <c r="Y6" s="25"/>
       <c r="Z6" s="25"/>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7" s="24"/>
       <c r="B7" s="24"/>
       <c r="C7" s="24"/>
@@ -1750,7 +1750,7 @@
       <c r="Y7" s="25"/>
       <c r="Z7" s="25"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8" s="24"/>
       <c r="B8" s="24"/>
       <c r="C8" s="24"/>
@@ -1778,7 +1778,7 @@
       <c r="Y8" s="25"/>
       <c r="Z8" s="25"/>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A9" s="24"/>
       <c r="B9" s="24"/>
       <c r="C9" s="24"/>
@@ -1806,7 +1806,7 @@
       <c r="Y9" s="25"/>
       <c r="Z9" s="25"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10" s="24"/>
       <c r="B10" s="24"/>
       <c r="C10" s="24"/>
@@ -1834,7 +1834,7 @@
       <c r="Y10" s="25"/>
       <c r="Z10" s="25"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A11" s="24"/>
       <c r="B11" s="24"/>
       <c r="C11" s="24"/>
@@ -1862,7 +1862,7 @@
       <c r="Y11" s="25"/>
       <c r="Z11" s="25"/>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A12" s="24"/>
       <c r="B12" s="24"/>
       <c r="C12" s="24"/>
@@ -1890,7 +1890,7 @@
       <c r="Y12" s="25"/>
       <c r="Z12" s="25"/>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A13" s="24"/>
       <c r="B13" s="24"/>
       <c r="C13" s="24"/>
@@ -1918,7 +1918,7 @@
       <c r="Y13" s="25"/>
       <c r="Z13" s="25"/>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A14" s="24"/>
       <c r="B14" s="24"/>
       <c r="C14" s="24"/>
@@ -1946,7 +1946,7 @@
       <c r="Y14" s="25"/>
       <c r="Z14" s="25"/>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A15" s="24"/>
       <c r="B15" s="24"/>
       <c r="C15" s="24"/>
@@ -1974,7 +1974,7 @@
       <c r="Y15" s="25"/>
       <c r="Z15" s="25"/>
     </row>
-    <row r="16" spans="1:26" ht="102.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:26" ht="102.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="40" t="s">
         <v>125</v>
       </c>
@@ -2004,7 +2004,7 @@
       <c r="Y16" s="25"/>
       <c r="Z16" s="25"/>
     </row>
-    <row r="17" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="28"/>
       <c r="B17" s="28"/>
       <c r="C17" s="28"/>
@@ -2032,7 +2032,7 @@
       <c r="Y17" s="25"/>
       <c r="Z17" s="25"/>
     </row>
-    <row r="18" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="28"/>
       <c r="B18" s="28"/>
       <c r="C18" s="28"/>
@@ -2060,7 +2060,7 @@
       <c r="Y18" s="25"/>
       <c r="Z18" s="25"/>
     </row>
-    <row r="19" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="31" t="s">
         <v>0</v>
       </c>
@@ -2092,7 +2092,7 @@
       <c r="Y19" s="25"/>
       <c r="Z19" s="25"/>
     </row>
-    <row r="20" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="31" t="s">
         <v>126</v>
       </c>
@@ -2124,7 +2124,7 @@
       <c r="Y20" s="25"/>
       <c r="Z20" s="25"/>
     </row>
-    <row r="21" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="31" t="s">
         <v>127</v>
       </c>
@@ -2156,7 +2156,7 @@
       <c r="Y21" s="25"/>
       <c r="Z21" s="25"/>
     </row>
-    <row r="22" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="31"/>
       <c r="B22" s="34"/>
       <c r="C22" s="34"/>
@@ -2184,7 +2184,7 @@
       <c r="Y22" s="25"/>
       <c r="Z22" s="25"/>
     </row>
-    <row r="23" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="31" t="s">
         <v>128</v>
       </c>
@@ -2216,7 +2216,7 @@
       <c r="Y23" s="25"/>
       <c r="Z23" s="25"/>
     </row>
-    <row r="24" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="31"/>
       <c r="B24" s="34" t="s">
         <v>140</v>
@@ -2246,7 +2246,7 @@
       <c r="Y24" s="25"/>
       <c r="Z24" s="25"/>
     </row>
-    <row r="25" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="31"/>
       <c r="B25" s="34"/>
       <c r="C25" s="34"/>
@@ -2274,7 +2274,7 @@
       <c r="Y25" s="25"/>
       <c r="Z25" s="25"/>
     </row>
-    <row r="26" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="31" t="s">
         <v>129</v>
       </c>
@@ -2306,7 +2306,7 @@
       <c r="Y26" s="25"/>
       <c r="Z26" s="25"/>
     </row>
-    <row r="27" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="31"/>
       <c r="B27" s="34"/>
       <c r="C27" s="34"/>
@@ -2334,7 +2334,7 @@
       <c r="Y27" s="25"/>
       <c r="Z27" s="25"/>
     </row>
-    <row r="28" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="31"/>
       <c r="B28" s="34"/>
       <c r="C28" s="34"/>
@@ -2362,7 +2362,7 @@
       <c r="Y28" s="25"/>
       <c r="Z28" s="25"/>
     </row>
-    <row r="29" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="31" t="s">
         <v>130</v>
       </c>
@@ -2394,7 +2394,7 @@
       <c r="Y29" s="25"/>
       <c r="Z29" s="25"/>
     </row>
-    <row r="30" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="31" t="s">
         <v>131</v>
       </c>
@@ -2426,7 +2426,7 @@
       <c r="Y30" s="25"/>
       <c r="Z30" s="25"/>
     </row>
-    <row r="31" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="31" t="s">
         <v>133</v>
       </c>
@@ -2458,7 +2458,7 @@
       <c r="Y31" s="25"/>
       <c r="Z31" s="25"/>
     </row>
-    <row r="32" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="37"/>
       <c r="B32" s="38" t="s">
         <v>135</v>
@@ -2488,7 +2488,7 @@
       <c r="Y32" s="25"/>
       <c r="Z32" s="25"/>
     </row>
-    <row r="33" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A33" s="24"/>
       <c r="B33" s="24"/>
       <c r="C33" s="24"/>
@@ -2516,7 +2516,7 @@
       <c r="Y33" s="25"/>
       <c r="Z33" s="25"/>
     </row>
-    <row r="34" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A34" s="24"/>
       <c r="B34" s="24"/>
       <c r="C34" s="24"/>
@@ -2544,7 +2544,7 @@
       <c r="Y34" s="25"/>
       <c r="Z34" s="25"/>
     </row>
-    <row r="35" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A35" s="24"/>
       <c r="B35" s="24"/>
       <c r="C35" s="24"/>
@@ -2572,7 +2572,7 @@
       <c r="Y35" s="25"/>
       <c r="Z35" s="25"/>
     </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A36" s="24"/>
       <c r="B36" s="24"/>
       <c r="C36" s="24"/>
@@ -2600,7 +2600,7 @@
       <c r="Y36" s="25"/>
       <c r="Z36" s="25"/>
     </row>
-    <row r="37" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A37" s="24"/>
       <c r="B37" s="24"/>
       <c r="C37" s="24"/>
@@ -2628,7 +2628,7 @@
       <c r="Y37" s="25"/>
       <c r="Z37" s="25"/>
     </row>
-    <row r="38" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A38" s="24"/>
       <c r="B38" s="24"/>
       <c r="C38" s="24"/>
@@ -2656,7 +2656,7 @@
       <c r="Y38" s="25"/>
       <c r="Z38" s="25"/>
     </row>
-    <row r="39" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="24"/>
@@ -2684,7 +2684,7 @@
       <c r="Y39" s="25"/>
       <c r="Z39" s="25"/>
     </row>
-    <row r="40" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A40" s="24"/>
       <c r="B40" s="24"/>
       <c r="C40" s="24"/>
@@ -2712,7 +2712,7 @@
       <c r="Y40" s="25"/>
       <c r="Z40" s="25"/>
     </row>
-    <row r="41" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A41" s="24"/>
       <c r="B41" s="24"/>
       <c r="C41" s="24"/>
@@ -2740,7 +2740,7 @@
       <c r="Y41" s="25"/>
       <c r="Z41" s="25"/>
     </row>
-    <row r="42" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A42" s="24"/>
       <c r="B42" s="24"/>
       <c r="C42" s="24"/>
@@ -2768,7 +2768,7 @@
       <c r="Y42" s="25"/>
       <c r="Z42" s="25"/>
     </row>
-    <row r="43" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A43" s="25"/>
       <c r="B43" s="25"/>
       <c r="C43" s="25"/>
@@ -2796,7 +2796,7 @@
       <c r="Y43" s="25"/>
       <c r="Z43" s="25"/>
     </row>
-    <row r="44" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A44" s="25"/>
       <c r="B44" s="25"/>
       <c r="C44" s="25"/>
@@ -2824,7 +2824,7 @@
       <c r="Y44" s="25"/>
       <c r="Z44" s="25"/>
     </row>
-    <row r="45" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A45" s="25"/>
       <c r="B45" s="25"/>
       <c r="C45" s="25"/>
@@ -2852,7 +2852,7 @@
       <c r="Y45" s="25"/>
       <c r="Z45" s="25"/>
     </row>
-    <row r="46" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A46" s="25"/>
       <c r="B46" s="25"/>
       <c r="C46" s="25"/>
@@ -2880,7 +2880,7 @@
       <c r="Y46" s="25"/>
       <c r="Z46" s="25"/>
     </row>
-    <row r="47" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A47" s="25"/>
       <c r="B47" s="25"/>
       <c r="C47" s="25"/>
@@ -2908,7 +2908,7 @@
       <c r="Y47" s="25"/>
       <c r="Z47" s="25"/>
     </row>
-    <row r="48" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A48" s="25"/>
       <c r="B48" s="25"/>
       <c r="C48" s="25"/>
@@ -2936,7 +2936,7 @@
       <c r="Y48" s="25"/>
       <c r="Z48" s="25"/>
     </row>
-    <row r="49" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A49" s="25"/>
       <c r="B49" s="25"/>
       <c r="C49" s="25"/>
@@ -2964,7 +2964,7 @@
       <c r="Y49" s="25"/>
       <c r="Z49" s="25"/>
     </row>
-    <row r="50" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A50" s="25"/>
       <c r="B50" s="25"/>
       <c r="C50" s="25"/>
@@ -2992,7 +2992,7 @@
       <c r="Y50" s="25"/>
       <c r="Z50" s="25"/>
     </row>
-    <row r="51" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A51" s="25"/>
       <c r="B51" s="25"/>
       <c r="C51" s="25"/>
@@ -3020,7 +3020,7 @@
       <c r="Y51" s="25"/>
       <c r="Z51" s="25"/>
     </row>
-    <row r="52" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A52" s="25"/>
       <c r="B52" s="25"/>
       <c r="C52" s="25"/>
@@ -3048,7 +3048,7 @@
       <c r="Y52" s="25"/>
       <c r="Z52" s="25"/>
     </row>
-    <row r="53" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A53" s="25"/>
       <c r="B53" s="25"/>
       <c r="C53" s="25"/>
@@ -3076,7 +3076,7 @@
       <c r="Y53" s="25"/>
       <c r="Z53" s="25"/>
     </row>
-    <row r="54" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A54" s="25"/>
       <c r="B54" s="25"/>
       <c r="C54" s="25"/>
@@ -3104,7 +3104,7 @@
       <c r="Y54" s="25"/>
       <c r="Z54" s="25"/>
     </row>
-    <row r="55" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A55" s="25"/>
       <c r="B55" s="25"/>
       <c r="C55" s="25"/>
@@ -3132,7 +3132,7 @@
       <c r="Y55" s="25"/>
       <c r="Z55" s="25"/>
     </row>
-    <row r="56" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A56" s="25"/>
       <c r="B56" s="25"/>
       <c r="C56" s="25"/>
@@ -3160,7 +3160,7 @@
       <c r="Y56" s="25"/>
       <c r="Z56" s="25"/>
     </row>
-    <row r="57" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A57" s="25"/>
       <c r="B57" s="25"/>
       <c r="C57" s="25"/>
@@ -3188,7 +3188,7 @@
       <c r="Y57" s="25"/>
       <c r="Z57" s="25"/>
     </row>
-    <row r="58" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A58" s="25"/>
       <c r="B58" s="25"/>
       <c r="C58" s="25"/>
@@ -3216,7 +3216,7 @@
       <c r="Y58" s="25"/>
       <c r="Z58" s="25"/>
     </row>
-    <row r="59" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A59" s="25"/>
       <c r="B59" s="25"/>
       <c r="C59" s="25"/>
@@ -3244,7 +3244,7 @@
       <c r="Y59" s="25"/>
       <c r="Z59" s="25"/>
     </row>
-    <row r="60" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A60" s="25"/>
       <c r="B60" s="25"/>
       <c r="C60" s="25"/>
@@ -3272,7 +3272,7 @@
       <c r="Y60" s="25"/>
       <c r="Z60" s="25"/>
     </row>
-    <row r="61" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A61" s="25"/>
       <c r="B61" s="25"/>
       <c r="C61" s="25"/>
@@ -3300,7 +3300,7 @@
       <c r="Y61" s="25"/>
       <c r="Z61" s="25"/>
     </row>
-    <row r="62" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A62" s="25"/>
       <c r="B62" s="25"/>
       <c r="C62" s="25"/>
@@ -3328,7 +3328,7 @@
       <c r="Y62" s="25"/>
       <c r="Z62" s="25"/>
     </row>
-    <row r="63" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A63" s="25"/>
       <c r="B63" s="25"/>
       <c r="C63" s="25"/>
@@ -3356,7 +3356,7 @@
       <c r="Y63" s="25"/>
       <c r="Z63" s="25"/>
     </row>
-    <row r="64" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A64" s="25"/>
       <c r="B64" s="25"/>
       <c r="C64" s="25"/>
@@ -3384,7 +3384,7 @@
       <c r="Y64" s="25"/>
       <c r="Z64" s="25"/>
     </row>
-    <row r="65" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A65" s="25"/>
       <c r="B65" s="25"/>
       <c r="C65" s="25"/>
@@ -3412,7 +3412,7 @@
       <c r="Y65" s="25"/>
       <c r="Z65" s="25"/>
     </row>
-    <row r="66" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A66" s="25"/>
       <c r="B66" s="25"/>
       <c r="C66" s="25"/>
@@ -3440,7 +3440,7 @@
       <c r="Y66" s="25"/>
       <c r="Z66" s="25"/>
     </row>
-    <row r="67" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A67" s="25"/>
       <c r="B67" s="25"/>
       <c r="C67" s="25"/>
@@ -3468,7 +3468,7 @@
       <c r="Y67" s="25"/>
       <c r="Z67" s="25"/>
     </row>
-    <row r="68" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A68" s="25"/>
       <c r="B68" s="25"/>
       <c r="C68" s="25"/>
@@ -3496,7 +3496,7 @@
       <c r="Y68" s="25"/>
       <c r="Z68" s="25"/>
     </row>
-    <row r="69" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A69" s="25"/>
       <c r="B69" s="25"/>
       <c r="C69" s="25"/>
@@ -3524,7 +3524,7 @@
       <c r="Y69" s="25"/>
       <c r="Z69" s="25"/>
     </row>
-    <row r="70" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A70" s="25"/>
       <c r="B70" s="25"/>
       <c r="C70" s="25"/>
@@ -3552,7 +3552,7 @@
       <c r="Y70" s="25"/>
       <c r="Z70" s="25"/>
     </row>
-    <row r="71" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A71" s="25"/>
       <c r="B71" s="25"/>
       <c r="C71" s="25"/>
@@ -3580,7 +3580,7 @@
       <c r="Y71" s="25"/>
       <c r="Z71" s="25"/>
     </row>
-    <row r="72" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A72" s="25"/>
       <c r="B72" s="25"/>
       <c r="C72" s="25"/>
@@ -3608,7 +3608,7 @@
       <c r="Y72" s="25"/>
       <c r="Z72" s="25"/>
     </row>
-    <row r="73" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A73" s="25"/>
       <c r="B73" s="25"/>
       <c r="C73" s="25"/>
@@ -3636,7 +3636,7 @@
       <c r="Y73" s="25"/>
       <c r="Z73" s="25"/>
     </row>
-    <row r="74" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A74" s="25"/>
       <c r="B74" s="25"/>
       <c r="C74" s="25"/>
@@ -3664,7 +3664,7 @@
       <c r="Y74" s="25"/>
       <c r="Z74" s="25"/>
     </row>
-    <row r="75" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A75" s="25"/>
       <c r="B75" s="25"/>
       <c r="C75" s="25"/>
@@ -3692,7 +3692,7 @@
       <c r="Y75" s="25"/>
       <c r="Z75" s="25"/>
     </row>
-    <row r="76" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A76" s="25"/>
       <c r="B76" s="25"/>
       <c r="C76" s="25"/>
@@ -3720,7 +3720,7 @@
       <c r="Y76" s="25"/>
       <c r="Z76" s="25"/>
     </row>
-    <row r="77" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A77" s="25"/>
       <c r="B77" s="25"/>
       <c r="C77" s="25"/>
@@ -3748,7 +3748,7 @@
       <c r="Y77" s="25"/>
       <c r="Z77" s="25"/>
     </row>
-    <row r="78" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A78" s="25"/>
       <c r="B78" s="25"/>
       <c r="C78" s="25"/>
@@ -3776,7 +3776,7 @@
       <c r="Y78" s="25"/>
       <c r="Z78" s="25"/>
     </row>
-    <row r="79" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A79" s="25"/>
       <c r="B79" s="25"/>
       <c r="C79" s="25"/>
@@ -3804,7 +3804,7 @@
       <c r="Y79" s="25"/>
       <c r="Z79" s="25"/>
     </row>
-    <row r="80" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A80" s="25"/>
       <c r="B80" s="25"/>
       <c r="C80" s="25"/>
@@ -3832,7 +3832,7 @@
       <c r="Y80" s="25"/>
       <c r="Z80" s="25"/>
     </row>
-    <row r="81" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A81" s="25"/>
       <c r="B81" s="25"/>
       <c r="C81" s="25"/>
@@ -3860,7 +3860,7 @@
       <c r="Y81" s="25"/>
       <c r="Z81" s="25"/>
     </row>
-    <row r="82" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A82" s="25"/>
       <c r="B82" s="25"/>
       <c r="C82" s="25"/>
@@ -3888,7 +3888,7 @@
       <c r="Y82" s="25"/>
       <c r="Z82" s="25"/>
     </row>
-    <row r="83" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A83" s="25"/>
       <c r="B83" s="25"/>
       <c r="C83" s="25"/>
@@ -3916,7 +3916,7 @@
       <c r="Y83" s="25"/>
       <c r="Z83" s="25"/>
     </row>
-    <row r="84" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A84" s="25"/>
       <c r="B84" s="25"/>
       <c r="C84" s="25"/>
@@ -3944,7 +3944,7 @@
       <c r="Y84" s="25"/>
       <c r="Z84" s="25"/>
     </row>
-    <row r="85" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A85" s="25"/>
       <c r="B85" s="25"/>
       <c r="C85" s="25"/>
@@ -3972,7 +3972,7 @@
       <c r="Y85" s="25"/>
       <c r="Z85" s="25"/>
     </row>
-    <row r="86" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A86" s="25"/>
       <c r="B86" s="25"/>
       <c r="C86" s="25"/>
@@ -4000,7 +4000,7 @@
       <c r="Y86" s="25"/>
       <c r="Z86" s="25"/>
     </row>
-    <row r="87" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A87" s="25"/>
       <c r="B87" s="25"/>
       <c r="C87" s="25"/>
@@ -4028,7 +4028,7 @@
       <c r="Y87" s="25"/>
       <c r="Z87" s="25"/>
     </row>
-    <row r="88" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A88" s="25"/>
       <c r="B88" s="25"/>
       <c r="C88" s="25"/>
@@ -4056,7 +4056,7 @@
       <c r="Y88" s="25"/>
       <c r="Z88" s="25"/>
     </row>
-    <row r="89" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A89" s="25"/>
       <c r="B89" s="25"/>
       <c r="C89" s="25"/>
@@ -4084,7 +4084,7 @@
       <c r="Y89" s="25"/>
       <c r="Z89" s="25"/>
     </row>
-    <row r="90" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A90" s="25"/>
       <c r="B90" s="25"/>
       <c r="C90" s="25"/>
@@ -4112,7 +4112,7 @@
       <c r="Y90" s="25"/>
       <c r="Z90" s="25"/>
     </row>
-    <row r="91" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A91" s="25"/>
       <c r="B91" s="25"/>
       <c r="C91" s="25"/>
@@ -4140,7 +4140,7 @@
       <c r="Y91" s="25"/>
       <c r="Z91" s="25"/>
     </row>
-    <row r="92" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A92" s="25"/>
       <c r="B92" s="25"/>
       <c r="C92" s="25"/>
@@ -4168,7 +4168,7 @@
       <c r="Y92" s="25"/>
       <c r="Z92" s="25"/>
     </row>
-    <row r="93" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A93" s="25"/>
       <c r="B93" s="25"/>
       <c r="C93" s="25"/>
@@ -4196,7 +4196,7 @@
       <c r="Y93" s="25"/>
       <c r="Z93" s="25"/>
     </row>
-    <row r="94" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A94" s="25"/>
       <c r="B94" s="25"/>
       <c r="C94" s="25"/>
@@ -4224,7 +4224,7 @@
       <c r="Y94" s="25"/>
       <c r="Z94" s="25"/>
     </row>
-    <row r="95" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A95" s="25"/>
       <c r="B95" s="25"/>
       <c r="C95" s="25"/>
@@ -4252,7 +4252,7 @@
       <c r="Y95" s="25"/>
       <c r="Z95" s="25"/>
     </row>
-    <row r="96" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A96" s="25"/>
       <c r="B96" s="25"/>
       <c r="C96" s="25"/>
@@ -4280,7 +4280,7 @@
       <c r="Y96" s="25"/>
       <c r="Z96" s="25"/>
     </row>
-    <row r="97" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A97" s="25"/>
       <c r="B97" s="25"/>
       <c r="C97" s="25"/>
@@ -4308,7 +4308,7 @@
       <c r="Y97" s="25"/>
       <c r="Z97" s="25"/>
     </row>
-    <row r="98" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A98" s="25"/>
       <c r="B98" s="25"/>
       <c r="C98" s="25"/>
@@ -4336,7 +4336,7 @@
       <c r="Y98" s="25"/>
       <c r="Z98" s="25"/>
     </row>
-    <row r="99" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A99" s="25"/>
       <c r="B99" s="25"/>
       <c r="C99" s="25"/>
@@ -4390,38 +4390,38 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A2:AE17"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.7265625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="56.7265625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="19.08984375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="24.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="9.26953125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.08984375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="12.7265625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="17.08984375" style="1" customWidth="1"/>
-    <col min="10" max="19" width="11.08984375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="33.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="19.109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="24.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="9.21875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="12.77734375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="17.109375" style="1" customWidth="1"/>
+    <col min="10" max="19" width="11.109375" style="1" customWidth="1"/>
     <col min="20" max="21" width="12" style="1" customWidth="1"/>
-    <col min="22" max="23" width="8.81640625" style="1"/>
-    <col min="24" max="24" width="13.7265625" style="1" customWidth="1"/>
+    <col min="22" max="23" width="8.77734375" style="1"/>
+    <col min="24" max="24" width="13.77734375" style="1" customWidth="1"/>
     <col min="25" max="25" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="68.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="16384" width="8.81640625" style="1"/>
+    <col min="26" max="26" width="68.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:31" ht="23.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
         <v>76</v>
       </c>
       <c r="B2" s="11"/>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>45</v>
       </c>
       <c r="B3" s="7"/>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" s="7"/>
       <c r="B4" s="7"/>
       <c r="D4" s="9" t="s">
@@ -4438,7 +4438,7 @@
       <c r="AD4" s="8"/>
       <c r="AE4" s="7"/>
     </row>
-    <row r="5" spans="1:31" ht="26" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:31" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A5" s="21" t="s">
         <v>26</v>
       </c>
@@ -4527,7 +4527,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:31" ht="78.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:31" ht="97.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>19</v>
       </c>
@@ -4586,7 +4586,7 @@
       <c r="AD6" s="18"/>
       <c r="AE6" s="18"/>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
         <v>55</v>
       </c>
@@ -4635,7 +4635,7 @@
       <c r="AD7" s="16"/>
       <c r="AE7" s="16"/>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
         <v>52</v>
       </c>
@@ -4671,7 +4671,7 @@
       <c r="AD8" s="13"/>
       <c r="AE8" s="13"/>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>51</v>
       </c>
@@ -4691,7 +4691,7 @@
         <v>30</v>
       </c>
       <c r="G9" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H9" s="1">
         <v>1</v>
@@ -4749,7 +4749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
@@ -4759,12 +4759,12 @@
       <c r="R10" s="2"/>
       <c r="S10" s="2"/>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
       <c r="S11"/>
       <c r="T11"/>
       <c r="U11"/>
     </row>
-    <row r="12" spans="1:31" ht="23.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:31" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
         <v>46</v>
       </c>
@@ -4794,7 +4794,7 @@
       <c r="Y12"/>
       <c r="Z12"/>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>45</v>
       </c>
@@ -4824,7 +4824,7 @@
       <c r="Y13"/>
       <c r="Z13"/>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" s="10"/>
       <c r="C14"/>
       <c r="D14" s="9" t="s">
@@ -4854,7 +4854,7 @@
       <c r="AD14" s="8"/>
       <c r="AE14" s="7"/>
     </row>
-    <row r="15" spans="1:31" ht="26" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:31" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>26</v>
       </c>
@@ -4929,7 +4929,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:31" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:31" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>19</v>
       </c>
@@ -4976,7 +4976,7 @@
       <c r="AD16" s="3"/>
       <c r="AE16" s="3"/>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>9</v>
       </c>
@@ -5051,32 +5051,32 @@
     <tabColor theme="7" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:X10"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.7265625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="29.26953125" style="1" customWidth="1"/>
-    <col min="3" max="5" width="12.81640625" style="1" customWidth="1"/>
-    <col min="6" max="8" width="8.81640625" style="1"/>
-    <col min="9" max="15" width="16.7265625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="8.81640625" style="1"/>
-    <col min="17" max="17" width="11.7265625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="11.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="29.21875" style="1" customWidth="1"/>
+    <col min="3" max="5" width="12.77734375" style="1" customWidth="1"/>
+    <col min="6" max="8" width="8.77734375" style="1"/>
+    <col min="9" max="15" width="16.77734375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="8.77734375" style="1"/>
+    <col min="17" max="17" width="11.77734375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="11.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="21" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="8.81640625" style="1"/>
+    <col min="20" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="23.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:24" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>95</v>
       </c>
       <c r="B1" s="11"/>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="E3" s="9" t="s">
         <v>44</v>
       </c>
@@ -5090,7 +5090,7 @@
       <c r="V3" s="8"/>
       <c r="W3" s="8"/>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4" s="21" t="s">
         <v>26</v>
       </c>
@@ -5161,7 +5161,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:24" ht="78.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:24" ht="83.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="19" t="s">
         <v>19</v>
       </c>
@@ -5216,7 +5216,7 @@
       <c r="W5" s="18"/>
       <c r="X5" s="18"/>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A6" s="16" t="s">
         <v>55</v>
       </c>
@@ -5259,7 +5259,7 @@
       <c r="W6" s="16"/>
       <c r="X6" s="16"/>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>82</v>
       </c>
@@ -5289,7 +5289,7 @@
       <c r="W7" s="13"/>
       <c r="X7" s="13"/>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>81</v>
       </c>
@@ -5353,7 +5353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>78</v>
       </c>
@@ -5361,7 +5361,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>78</v>
       </c>
@@ -5387,30 +5387,30 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:Z10"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" style="1" customWidth="1"/>
-    <col min="2" max="2" width="57.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12.36328125" style="1" customWidth="1"/>
-    <col min="5" max="17" width="14.26953125" style="1" customWidth="1"/>
-    <col min="18" max="19" width="8.81640625" style="1"/>
-    <col min="20" max="20" width="11.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="56.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="16384" width="8.81640625" style="1"/>
+    <col min="2" max="2" width="57.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="12.33203125" style="1" customWidth="1"/>
+    <col min="5" max="17" width="14.21875" style="1" customWidth="1"/>
+    <col min="18" max="19" width="8.77734375" style="1"/>
+    <col min="20" max="20" width="11.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="56.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="23.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:26" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>111</v>
       </c>
       <c r="B1" s="11"/>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="D3" s="9" t="s">
         <v>141</v>
       </c>
@@ -5424,7 +5424,7 @@
       <c r="X3" s="8"/>
       <c r="Y3" s="8"/>
     </row>
-    <row r="4" spans="1:26" ht="26" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:26" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A4" s="21" t="s">
         <v>26</v>
       </c>
@@ -5501,7 +5501,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:26" ht="91.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:26" ht="111" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="19" t="s">
         <v>19</v>
       </c>
@@ -5564,7 +5564,7 @@
       <c r="Y5" s="18"/>
       <c r="Z5" s="18"/>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:26" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A6" s="16" t="s">
         <v>55</v>
       </c>
@@ -5613,7 +5613,7 @@
       <c r="Y6" s="16"/>
       <c r="Z6" s="16"/>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>103</v>
       </c>
@@ -5645,7 +5645,7 @@
       <c r="Y7" s="13"/>
       <c r="Z7" s="13"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>102</v>
       </c>
@@ -5714,7 +5714,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>100</v>
       </c>
@@ -5781,7 +5781,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>97</v>
       </c>
@@ -5859,36 +5859,36 @@
     <tabColor theme="5" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:V8"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.7265625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.36328125" style="1" customWidth="1"/>
-    <col min="5" max="8" width="8.81640625" style="1"/>
-    <col min="9" max="9" width="14.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.7265625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="6.36328125" customWidth="1"/>
-    <col min="13" max="13" width="11.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="23.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="21" width="8.81640625" style="1"/>
-    <col min="22" max="22" width="2.7265625" customWidth="1"/>
-    <col min="23" max="16384" width="8.81640625" style="1"/>
+    <col min="1" max="1" width="17.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.33203125" style="1" customWidth="1"/>
+    <col min="5" max="8" width="8.77734375" style="1"/>
+    <col min="9" max="9" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.77734375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="6.33203125" customWidth="1"/>
+    <col min="13" max="13" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="23.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="21" width="8.77734375" style="1"/>
+    <col min="22" max="22" width="2.77734375" customWidth="1"/>
+    <col min="23" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="23.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:20" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>124</v>
       </c>
       <c r="B1" s="11"/>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="D3" s="9" t="s">
         <v>44</v>
       </c>
@@ -5902,7 +5902,7 @@
       <c r="R3" s="8"/>
       <c r="S3" s="8"/>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" s="21" t="s">
         <v>26</v>
       </c>
@@ -5961,7 +5961,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:20" ht="47.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:20" ht="47.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="19" t="s">
         <v>19</v>
       </c>
@@ -6004,7 +6004,7 @@
       <c r="S5" s="18"/>
       <c r="T5" s="18"/>
     </row>
-    <row r="6" spans="1:20" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:20" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="16" t="s">
         <v>55</v>
       </c>
@@ -6037,7 +6037,7 @@
       <c r="S6" s="16"/>
       <c r="T6" s="16"/>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>117</v>
       </c>
@@ -6095,7 +6095,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>115</v>
       </c>

</xml_diff>